<commit_message>
Atualização automática: reajuste (16/07/2026 20:17)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (22/07/2026 12:04)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (22/07/2026 16:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (23/07/2026 11:42)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (23/07/2026 16:18)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (18/08/2026 12:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (18/08/2026 12:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (19/08/2026 13:09)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (19/08/2026 14:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (21/08/2026 09:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (21/08/2026 10:53)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (24/08/2026 12:50)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -1012,18 +1012,18 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B33" t="s">
         <v>27</v>
       </c>
       <c r="C33">
-        <v>9226114.959000001</v>
+        <v>9268344.682</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B34" t="s">
         <v>3</v>
@@ -1034,18 +1034,18 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
       </c>
       <c r="C35">
-        <v>27227.68</v>
+        <v>69457.40325</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B36" t="s">
         <v>5</v>
@@ -1056,7 +1056,7 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B37" t="s">
         <v>28</v>
@@ -1067,18 +1067,18 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B38" t="s">
         <v>29</v>
       </c>
       <c r="C38">
-        <v>509263.9148</v>
+        <v>467034.1916</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B39" t="s">
         <v>30</v>
@@ -1089,18 +1089,18 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
         <v>31</v>
       </c>
       <c r="C40">
-        <v>76936421.59</v>
+        <v>76894191.87</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B41" t="s">
         <v>12</v>
@@ -1111,7 +1111,7 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B42" t="s">
         <v>13</v>
@@ -1122,7 +1122,7 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B43" t="s">
         <v>14</v>
@@ -1133,7 +1133,7 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B44" t="s">
         <v>15</v>
@@ -1144,7 +1144,7 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B45" t="s">
         <v>16</v>
@@ -1155,7 +1155,7 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B46" t="s">
         <v>17</v>
@@ -1166,7 +1166,7 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B47" t="s">
         <v>18</v>
@@ -1177,7 +1177,7 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B48" t="s">
         <v>32</v>
@@ -1188,18 +1188,18 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B49" t="s">
         <v>33</v>
       </c>
       <c r="C49">
-        <v>509263.9148</v>
+        <v>467034.1916</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B50" t="s">
         <v>34</v>
@@ -1210,18 +1210,18 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B51" t="s">
         <v>35</v>
       </c>
       <c r="C51">
-        <v>76936421.59</v>
+        <v>76894191.87</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B52" t="s">
         <v>36</v>
@@ -1232,7 +1232,7 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B53" t="s">
         <v>24</v>
@@ -1243,7 +1243,7 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B54" t="s">
         <v>25</v>
@@ -1254,7 +1254,7 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B55" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Atualização automática: reajuste (25/08/2026 08:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (25/08/2026 08:37)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (01/09/2026 11:17)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (01/09/2026 12:29)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (02/09/2026 09:40)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (02/09/2026 12:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (03/09/2026 13:44)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (04/09/2026 11:56)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (08/09/2026 08:24)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (08/09/2026 12:05)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>